<commit_message>
Cache formula results in shipment summary workbook
LibreOffice cannot run in this environment, so the usual recalculation step
could not populate cached values and every total read back as empty in any
reader that relies on them.

Evaluate the SUM/SUMIF totals from the Detail sheet's literal cells and write
them into the sheet XML as cached results, keeping the formulas themselves
intact, and set fullCalcOnLoad so Excel still recalculates on open.

Co-Authored-By: Claude Opus 5 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_019yHzjMmDQHFt3y1UvA2qQh
</commit_message>
<xml_diff>
--- a/output/Summary_Sunking_Pacific_2026-08-12.xlsx
+++ b/output/Summary_Sunking_Pacific_2026-08-12.xlsx
@@ -676,11 +676,11 @@
       </c>
       <c r="C5" s="6">
         <f>SUMIF(Detail!$A$6:$A$10,$A5,Detail!$G$6:$G$10)</f>
-        <v/>
+        <v>651</v>
       </c>
       <c r="D5" s="7">
         <f>SUMIF(Detail!$A$6:$A$10,$A5,Detail!$H$6:$H$10)</f>
-        <v/>
+        <v>2213.4</v>
       </c>
       <c r="E5" s="8" t="inlineStr">
         <is>
@@ -706,11 +706,11 @@
       </c>
       <c r="C6" s="6">
         <f>SUMIF(Detail!$A$6:$A$10,$A6,Detail!$G$6:$G$10)</f>
-        <v/>
+        <v>256</v>
       </c>
       <c r="D6" s="7">
         <f>SUMIF(Detail!$A$6:$A$10,$A6,Detail!$H$6:$H$10)</f>
-        <v/>
+        <v>665.6</v>
       </c>
       <c r="E6" s="8" t="inlineStr">
         <is>
@@ -736,11 +736,11 @@
       </c>
       <c r="C7" s="6">
         <f>SUMIF(Detail!$A$6:$A$10,$A7,Detail!$G$6:$G$10)</f>
-        <v/>
+        <v>64</v>
       </c>
       <c r="D7" s="7">
         <f>SUMIF(Detail!$A$6:$A$10,$A7,Detail!$H$6:$H$10)</f>
-        <v/>
+        <v>192</v>
       </c>
       <c r="E7" s="8" t="inlineStr">
         <is>
@@ -762,11 +762,11 @@
       <c r="B8" s="11" t="n"/>
       <c r="C8" s="12">
         <f>SUM(C5:C7)</f>
-        <v/>
+        <v>971</v>
       </c>
       <c r="D8" s="13">
         <f>SUM(D5:D7)</f>
-        <v/>
+        <v>3071</v>
       </c>
       <c r="E8" s="10" t="inlineStr">
         <is>
@@ -1113,11 +1113,11 @@
       <c r="F11" s="26" t="n"/>
       <c r="G11" s="27">
         <f>SUM(G6:G10)</f>
-        <v/>
+        <v>971</v>
       </c>
       <c r="H11" s="28">
         <f>SUM(H6:H10)</f>
-        <v/>
+        <v>3071</v>
       </c>
       <c r="I11" s="26" t="n"/>
     </row>

</xml_diff>